<commit_message>
Debugged extra underscore issue in cancer type
</commit_message>
<xml_diff>
--- a/b_cancer_incidence/cancer_type_radiotherapy.xlsx
+++ b/b_cancer_incidence/cancer_type_radiotherapy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiamartin/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alikaho/Desktop/STELLA/Geospatial-modelling-radiotherapy-access/b_cancer_incidence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C19482-9118-E145-A34C-9418CBE47C81}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAB6AE6-0263-AE41-88C8-3C3A0419105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3080" yWindow="2060" windowWidth="28040" windowHeight="17440" xr2:uid="{FB5A2ABA-A8C1-EC43-AF24-0D9F90F3EE26}"/>
+    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="16860" xr2:uid="{FB5A2ABA-A8C1-EC43-AF24-0D9F90F3EE26}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,15 +48,9 @@
     <t>Prostate</t>
   </si>
   <si>
-    <t xml:space="preserve">Bowel </t>
-  </si>
-  <si>
     <t>Lung</t>
   </si>
   <si>
-    <t xml:space="preserve">Non-Hodgkins lymphoma </t>
-  </si>
-  <si>
     <t>Kidney</t>
   </si>
   <si>
@@ -72,16 +66,22 @@
     <t>Uterus</t>
   </si>
   <si>
-    <t xml:space="preserve">Ovary </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other </t>
-  </si>
-  <si>
     <t>fraction</t>
   </si>
   <si>
     <t>proportion of cases</t>
+  </si>
+  <si>
+    <t>Bowel</t>
+  </si>
+  <si>
+    <t>Non-Hodgkins lymphoma</t>
+  </si>
+  <si>
+    <t>Ovary</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -138,9 +138,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -178,7 +178,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -284,7 +284,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -426,7 +426,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -447,13 +447,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -486,7 +486,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>0.126</v>
@@ -500,7 +500,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>0.124</v>
@@ -514,7 +514,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>3.4000000000000002E-2</v>
@@ -528,7 +528,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>3.1E-2</v>
@@ -542,7 +542,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>2.9000000000000001E-2</v>
@@ -556,7 +556,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>2.8000000000000001E-2</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10">
         <v>2.8000000000000001E-2</v>
@@ -584,7 +584,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>2.69E-2</v>
@@ -598,7 +598,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1.7899999999999999E-2</v>
@@ -612,7 +612,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.2263</v>

</xml_diff>

<commit_message>
now has option to run optimally treated
</commit_message>
<xml_diff>
--- a/b_cancer_incidence/cancer_type_radiotherapy.xlsx
+++ b/b_cancer_incidence/cancer_type_radiotherapy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alikaho/Desktop/STELLA/Geospatial-modelling-radiotherapy-access/b_cancer_incidence/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiamartin/Desktop/src/b_cancer_incidence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAB6AE6-0263-AE41-88C8-3C3A0419105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4ED41C3-978A-F142-85D7-24E7875B76C7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="16860" xr2:uid="{FB5A2ABA-A8C1-EC43-AF24-0D9F90F3EE26}"/>
+    <workbookView xWindow="8520" yWindow="780" windowWidth="20280" windowHeight="16860" xr2:uid="{FB5A2ABA-A8C1-EC43-AF24-0D9F90F3EE26}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">Cancer Type </t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optimal fraction </t>
   </si>
 </sst>
 </file>
@@ -138,9 +141,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -178,7 +181,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -284,7 +287,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -426,7 +429,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -434,15 +437,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99C3D4F5-9A39-8F44-8430-05974A2CBE95}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="36.6640625" customWidth="1"/>
     <col min="3" max="3" width="52.33203125" customWidth="1"/>
     <col min="4" max="4" width="57.6640625" customWidth="1"/>
+    <col min="5" max="5" width="39.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -455,8 +459,11 @@
       <c r="D1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -469,8 +476,11 @@
       <c r="D2">
         <v>0.61799999999999999</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -483,8 +493,11 @@
       <c r="D3">
         <v>0.32600000000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -497,8 +510,11 @@
       <c r="D4">
         <v>0.129</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -511,8 +527,11 @@
       <c r="D5">
         <v>0.252</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -525,8 +544,11 @@
       <c r="D6">
         <v>0.433</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -539,8 +561,11 @@
       <c r="D7">
         <v>7.0999999999999994E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -553,8 +578,11 @@
       <c r="D8">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -567,8 +595,11 @@
       <c r="D9">
         <v>0.64</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -581,8 +612,11 @@
       <c r="D10">
         <v>2.5000000000000001E-2</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -595,8 +629,11 @@
       <c r="D11">
         <v>0.30499999999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E11">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -609,8 +646,11 @@
       <c r="D12">
         <v>1.7000000000000001E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E12">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -622,6 +662,9 @@
       </c>
       <c r="D13">
         <v>0.25700000000000001</v>
+      </c>
+      <c r="E13">
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>